<commit_message>
Validate complete renv environment lock
</commit_message>
<xml_diff>
--- a/PLOS_code_availability_checklist.xlsx
+++ b/PLOS_code_availability_checklist.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R13b02d9ceaa541ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R2aaa95eba6924f61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf825332c0a324042"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R6f160593dc604d9d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -495,7 +495,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
-        <x:v>The local package remains NOT READY because the dependency lock, verified remote, immutable tag, and Zenodo DOI are incomplete.</x:v>
+        <x:v>The local package remains NOT READY because final public-release authorization, an immutable tag, and a real Zenodo DOI are still pending.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -511,7 +511,7 @@
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="28" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="10" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="38" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="38" hidden="0" customWidth="1"/>
   </x:cols>
@@ -530,21 +530,21 @@
         <x:v>required_action</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="36" hidden="0" customHeight="1">
+    <x:row r="2" ht="48" hidden="0" customHeight="1">
       <x:c r="A2" s="31" t="str">
-        <x:v>Public repository</x:v>
+        <x:v>GitHub repository</x:v>
       </x:c>
       <x:c r="B2" s="31" t="str">
-        <x:v>FAIL</x:v>
+        <x:v>PASS WITH LIMITATION</x:v>
       </x:c>
       <x:c r="C2" s="31" t="str">
-        <x:v>Target owner/name supplied; unauthenticated GitHub API returned 404 and cannot verify a public or private remote</x:v>
+        <x:v>Local origin uses the owner-confirmed URL; owner reports the private repository was created and the initial commit was pushed; automated read-only verification ended with a connection reset</x:v>
       </x:c>
       <x:c r="D2" s="31" t="str">
-        <x:v>Create or authenticate and independently verify the remote</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3" ht="24" hidden="0" customHeight="1">
+        <x:v>Confirm the post-validation push in the web interface and verify public access before publication</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="36" hidden="0" customHeight="1">
       <x:c r="A3" s="32" t="str">
         <x:v>README</x:v>
       </x:c>
@@ -552,10 +552,10 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C3" s="32" t="str">
-        <x:v>Overview, accessions, structure, requirements, workflow, figures, limits, and license documented</x:v>
+        <x:v>Overview, accessions, structure, requirements, workflow, figures, limits, environment validation, private-remote status, and license documented</x:v>
       </x:c>
       <x:c r="D3" s="32" t="str">
-        <x:v>Update remote/DOI wording only after verification</x:v>
+        <x:v>Insert the real Zenodo DOI after archiving the tagged release</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="24" hidden="0" customHeight="1">
@@ -580,24 +580,24 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C5" s="32" t="str">
-        <x:v>Valid YAML/JSON; title, version 1.0.0, authors, and MIT license synchronized; DOI/ORCID/email/repository-code omitted</x:v>
+        <x:v>Valid YAML/JSON; title, version 1.0.0, authors, and MIT license synchronized; owner-confirmed repository URL recorded; DOI/ORCID/email omitted</x:v>
       </x:c>
       <x:c r="D5" s="32" t="str">
-        <x:v>Insert verified identifiers only after release</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="24" hidden="0" customHeight="1">
+        <x:v>Insert the real DOI only after release archival</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="48" hidden="0" customHeight="1">
       <x:c r="A6" s="32" t="str">
         <x:v>Environment lock</x:v>
       </x:c>
       <x:c r="B6" s="32" t="str">
-        <x:v>FAIL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="C6" s="32" t="str">
-        <x:v>renv.lock parses but contains zero packages; restore is a no-op; status reports project not using renv</x:v>
+        <x:v>188-package R 4.5.2/Bioconductor 3.22 lock; non-no-op sandboxed clean-project restore; zero missing packages and version mismatches; clean renv::status()</x:v>
       </x:c>
       <x:c r="D6" s="32" t="str">
-        <x:v>Generate and clean-restore a complete lock</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="24" hidden="0" customHeight="1">
@@ -670,7 +670,7 @@
         <x:v>None</x:v>
       </x:c>
     </x:row>
-    <x:row r="12" ht="24" hidden="0" customHeight="1">
+    <x:row r="12" ht="36" hidden="0" customHeight="1">
       <x:c r="A12" s="32" t="str">
         <x:v>Package versions</x:v>
       </x:c>
@@ -678,10 +678,10 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C12" s="32" t="str">
-        <x:v>22/22 recorded packages installed at canonical recorded versions in audit environment</x:v>
+        <x:v>22/22 declared direct/supporting packages and the 188-record dependency closure reconcile at the locked versions</x:v>
       </x:c>
       <x:c r="D12" s="32" t="str">
-        <x:v>Capture them in a complete renv.lock</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0" customHeight="1">
@@ -706,7 +706,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rec1c18c5a6ff406f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda70fd5a079c425f"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
Synchronize public release and DOI metadata
</commit_message>
<xml_diff>
--- a/PLOS_code_availability_checklist.xlsx
+++ b/PLOS_code_availability_checklist.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf825332c0a324042"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R6f160593dc604d9d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R331033187cf74463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checklist" sheetId="2" r:id="R59c218486ad649a5"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="7">
+  <x:fonts count="8">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -54,8 +54,14 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Calibri"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF006100"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="5">
+  <x:fills count="10">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -75,6 +81,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FFFDEDEC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFE2F0D9"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -132,7 +163,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="34">
+  <x:cellXfs count="40">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -203,6 +234,12 @@
     <x:xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="3" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -214,7 +251,7 @@
         <x:color rgb="FF1B7837"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE8F5E9"/>
         </x:patternFill>
       </x:fill>
@@ -225,7 +262,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDEDEC"/>
         </x:patternFill>
       </x:fill>
@@ -235,7 +272,7 @@
         <x:color rgb="FF9B1C1C"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDEDEC"/>
         </x:patternFill>
       </x:fill>
@@ -466,14 +503,15 @@
       <x:c r="E1" s="3"/>
       <x:c r="F1" s="3"/>
     </x:row>
-    <x:row r="3">
+    <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="5" t="str">
         <x:v>Overall status</x:v>
       </x:c>
-      <x:c r="B3" s="7" t="str">
-        <x:v>NOT READY</x:v>
-      </x:c>
-    </x:row>
+      <x:c r="B3" s="39" t="str">
+        <x:v>PUBLIC RELEASE AVAILABLE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4"/>
     <x:row r="5" ht="15" hidden="0" customHeight="1">
       <x:c r="A5" s="9" t="n">
         <x:v>1</x:v>
@@ -495,7 +533,7 @@
         <x:v>3</x:v>
       </x:c>
       <x:c r="B7" s="11" t="str">
-        <x:v>The local package remains NOT READY because final public-release authorization, an immutable tag, and a real Zenodo DOI are still pending.</x:v>
+        <x:v>The public repository, immutable v1.0.0 release, and verified Zenodo version and concept DOIs are available; scientific results remain locked.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -530,18 +568,18 @@
         <x:v>required_action</x:v>
       </x:c>
     </x:row>
-    <x:row r="2" ht="48" hidden="0" customHeight="1">
+    <x:row r="2" ht="36" hidden="0" customHeight="1">
       <x:c r="A2" s="31" t="str">
         <x:v>GitHub repository</x:v>
       </x:c>
       <x:c r="B2" s="31" t="str">
-        <x:v>PASS WITH LIMITATION</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="C2" s="31" t="str">
-        <x:v>Local origin uses the owner-confirmed URL; owner reports the private repository was created and the initial commit was pushed; automated read-only verification ended with a connection reset</x:v>
+        <x:v>Public repository verified at https://github.com/shice951229-oss/cross-tissue-module-reproducibility; v1.0.0 points to commit 3eb6474</x:v>
       </x:c>
       <x:c r="D2" s="31" t="str">
-        <x:v>Confirm the post-validation push in the web interface and verify public access before publication</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="36" hidden="0" customHeight="1">
@@ -552,13 +590,13 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C3" s="32" t="str">
-        <x:v>Overview, accessions, structure, requirements, workflow, figures, limits, environment validation, private-remote status, and license documented</x:v>
+        <x:v>Overview, public repository, release tag, version DOI, concept DOI, workflow, limits, environment validation, and license documented</x:v>
       </x:c>
       <x:c r="D3" s="32" t="str">
-        <x:v>Insert the real Zenodo DOI after archiving the tagged release</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="24" hidden="0" customHeight="1">
+        <x:v>None</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="36" hidden="0" customHeight="1">
       <x:c r="A4" s="32" t="str">
         <x:v>License</x:v>
       </x:c>
@@ -566,10 +604,10 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C4" s="32" t="str">
-        <x:v>MIT License applies only to author-generated code and documentation</x:v>
+        <x:v>MIT License applies only to author-generated code and documentation; author and institutional authorization confirmed</x:v>
       </x:c>
       <x:c r="D4" s="32" t="str">
-        <x:v>Final author and institutional authorization</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="36" hidden="0" customHeight="1">
@@ -580,10 +618,10 @@
         <x:v>PASS</x:v>
       </x:c>
       <x:c r="C5" s="32" t="str">
-        <x:v>Valid YAML/JSON; title, version 1.0.0, authors, and MIT license synchronized; owner-confirmed repository URL recorded; DOI/ORCID/email omitted</x:v>
+        <x:v>Valid YAML/JSON; title, version 1.0.0, authors, MIT license, public repository URL, and verified version DOI 10.5281/zenodo.21762839 synchronized</x:v>
       </x:c>
       <x:c r="D5" s="32" t="str">
-        <x:v>Insert the real DOI only after release archival</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" hidden="0" customHeight="1">
@@ -684,18 +722,18 @@
         <x:v>None</x:v>
       </x:c>
     </x:row>
-    <x:row r="13" ht="15" hidden="0" customHeight="1">
+    <x:row r="13" ht="36" hidden="0" customHeight="1">
       <x:c r="A13" s="33" t="str">
         <x:v>DOI archive</x:v>
       </x:c>
       <x:c r="B13" s="33" t="str">
-        <x:v>FAIL</x:v>
+        <x:v>PASS</x:v>
       </x:c>
       <x:c r="C13" s="33" t="str">
-        <x:v>No Zenodo DOI has been issued</x:v>
+        <x:v>Zenodo version DOI 10.5281/zenodo.21762839 archives v1.0.0; concept DOI 10.5281/zenodo.21762838 represents all versions</x:v>
       </x:c>
       <x:c r="D13" s="33" t="str">
-        <x:v>Archive an eligible immutable tag and insert the DOI</x:v>
+        <x:v>None</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -706,7 +744,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rda70fd5a079c425f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf9db747e23e34191"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>